<commit_message>
docs(sprint13): close pending Sprint 13 documentation deliverables
Adds a dedicated OpenAPI 3.0 spec for the MINSA/DIRESA/SINADEF institutional
API, updates README/ROADMAP docs and the traceability matrix (RF-002,
RF-005, RF-007, RF-008, RF-009) with the Sprint 13 scope, and marks the
Sprint 13 plan's own documentation deliverable as completed (6/6, closed).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/trazabilidad/Matriz_Trazabilidad_RespiCare.xlsx
+++ b/Documentation/trazabilidad/Matriz_Trazabilidad_RespiCare.xlsx
@@ -821,7 +821,9 @@
 Servicio de IA (ai-services, Python/FastAPI):
 • main.py — endpoint /api/v1/ml-analyze
 • ml_models/random_forest_model.py, xgboost_model.py, neural_network_model.py
-• shap_explainer.py — explicabilidad (RF-006)</t>
+• shap_explainer.py — explicabilidad (RF-006)
+Sprint 13 — API institucional (MINSA/DIRESA/SINADEF):
+• backend/src/services/institutionalIntegrationService.ts — getEpidemiologicalExport() reutiliza la analítica de tendencias/brotes ya generada a partir de estas predicciones, agregada por distrito, para el consumidor externo (backend/openapi/institutional-api.yaml)</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1337,10 @@
 • MedicalValidationRules (services/medical_validation_rules.py) — validation_rules, validate_prediction(disease, symptoms, age)
 • _apply_medical_validation(response, symptoms_str, patient_age) (api/routes/symptom_ml_analyzer.py) — aplica la validación y ajusta confidence/is_clinically_coherent/coherence_warnings en las 3 rutas de predicción de /v1/ml-analyze (ensemble, fallback SHAP, fallback por patrones)
 • BaseRandomForestModel (scripts/training/train_base_model.py) — compone validation_system (MedicalValidationRules, importado desde services/) y emergency_system (EmergencyRuleSystem)
-• HybridRuleMLSystem (hybrid_system.py) — permanece como código no utilizado por ninguna ruta de la API</t>
+• HybridRuleMLSystem (hybrid_system.py) — permanece como código no utilizado por ninguna ruta de la API
+Sprint 13 — validación de vitales de wearables:
+• MedicalValidationRules.validate_vitals(vitals) (services/medical_validation_rules.py) — umbrales clínicos para SpO2, frecuencia respiratoria y frecuencia cardíaca capturados por wearables cerca del reporte de síntomas; ajusta confidence_adjustment y puede activar urgency_escalation sin reemplazar el modelo de ML
+• backend/src/services/wearableService.ts — sincroniza y valida los datos crudos de wearables (BLE, Health Connect, HealthKit) antes de que lleguen a esta capa</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1685,11 @@
 • backend/src/models/AIAnalysis.ts — subdocumento review (status pending/approved/rejected/adjusted, doctorId, doctorName, comments, adjustedDiagnosis, adjustedUrgency, signature{signatureData, signatureMethod, signedAt}) y métodos approve()/reject()/adjust()
 • backend/src/services/aiAnalysisReviewService.ts — reviewPrediction() (valida al médico, evita doble revisión, notifica al paciente)
 • backend/src/routes/aiAnalysisReviewRoutes.ts — GET /pending, GET /:id, POST /:id/review (authorize('doctor','admin'))
-• backend/src/controllers/symptomAnalyzerController.ts — analyzeSymptomsML ahora persiste cada predicción real de /v1/ml-analyze como documento AIAnalysis, cerrando también la brecha de que ninguna predicción real llegaba a persistirse</t>
+• backend/src/controllers/symptomAnalyzerController.ts — analyzeSymptomsML ahora persiste cada predicción real de /v1/ml-analyze como documento AIAnalysis, cerrando también la brecha de que ninguna predicción real llegaba a persistirse
+Sprint 13 — Panel del médico rediseñado (clasificación clínica de 4 niveles: crítico/alto/medio/bajo):
+• web/src/pages/PatientMonitoringPage.js — stat-cards, tabla de pacientes bajo seguimiento, gráfico de tendencia SpO2 de 7 días (datos de wearables), feed de últimas alertas
+• web/src/pages/PatientMonitoringPage.css
+• web/src/pages/MedicalHistoryPage.js — soporta ?patientId= para el botón "Ver ficha" desde el panel</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1861,9 @@
 • controllers/medicalHistoryController.ts e interface-adapters/controllers/MedicalHistoryController.ts
 • routes/medicalHistoryRoutes.ts e interface-adapters/routes/MedicalHistoryRoutes.ts
 BD y modelos:
-• models/MedicalHistory.ts — esquema Mongoose del historial clínico</t>
+• models/MedicalHistory.ts — esquema Mongoose del historial clínico
+Sprint 13 — corrección de filtrado por médico:
+• backend/src/dev/medicalHistoriesDev.ts — GET /api/v1/medical-histories filtra correctamente por doctorId cuando el rol autenticado es "doctor" (antes filtraba por patientId=id del propio médico, devolviendo siempre 0 resultados)</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2037,9 @@
 • jobs/alertJobs.ts — scheduledQueueInterval / pendingAlertInterval
 • controllers/alertController.ts, routes/alertRoutes.ts
 BD y modelos:
-• models/Alert.ts — esquema Mongoose de la colección “alerts” (AlertPriority, AlertCategory, AlertStatus)</t>
+• models/Alert.ts — esquema Mongoose de la colección “alerts” (AlertPriority, AlertCategory, AlertStatus)
+Sprint 13 — alertas sanitarias institucionales (MINSA/SINADEF):
+• backend/src/services/institutionalIntegrationService.ts — ingestExternalAlert() crea un Alert (categoría health_authority) por cada médico/admin activo a partir de una alerta regional recibida vía POST /api/v1/institutional/alerts</t>
         </is>
       </c>
     </row>

</xml_diff>